<commit_message>
V3 WIP snapshot: in-flight agent work
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MjSxEeBc788vmeDLxVaq4s
</commit_message>
<xml_diff>
--- a/tests/fixtures/source/atlas.idmc/e092018d9e99cec1.xlsx
+++ b/tests/fixtures/source/atlas.idmc/e092018d9e99cec1.xlsx
@@ -716,6 +716,374 @@
       <c r="K6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
     </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>PHL</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Philippines: Storm - 01/01/2008</t>
+        </is>
+      </c>
+      <c r="E149" s="1" t="n">
+        <v>39448</v>
+      </c>
+      <c r="F149" t="n">
+        <v>2039000</v>
+      </c>
+      <c r="G149" t="n">
+        <v>2039155</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr"/>
+      <c r="M149" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>BEN</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Benin</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Benin: Flood - 01/01/2009</t>
+        </is>
+      </c>
+      <c r="E194" s="1" t="n">
+        <v>39814</v>
+      </c>
+      <c r="F194" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G194" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr"/>
+      <c r="M194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>BEN</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Benin</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Benin: Flood - 01/01/2009</t>
+        </is>
+      </c>
+      <c r="E195" s="1" t="n">
+        <v>39814</v>
+      </c>
+      <c r="F195" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G195" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Cyclone 'aila'</t>
+        </is>
+      </c>
+      <c r="E198" s="1" t="n">
+        <v>39814</v>
+      </c>
+      <c r="F198" t="n">
+        <v>842000</v>
+      </c>
+      <c r="G198" t="n">
+        <v>842000</v>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr"/>
+      <c r="M198" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Cyclone 'aila'</t>
+        </is>
+      </c>
+      <c r="E240" s="1" t="n">
+        <v>39814</v>
+      </c>
+      <c r="F240" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="G240" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr"/>
+      <c r="M240" t="inlineStr"/>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C650" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>United Kingdom: Flood - 01/01/2012</t>
+        </is>
+      </c>
+      <c r="E650" s="1" t="n">
+        <v>40909</v>
+      </c>
+      <c r="F650" t="n">
+        <v>100</v>
+      </c>
+      <c r="G650" t="n">
+        <v>100</v>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="K650" t="inlineStr"/>
+      <c r="M650" t="inlineStr"/>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C651" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>United Kingdom: Flood - 01/01/2012</t>
+        </is>
+      </c>
+      <c r="E651" s="1" t="n">
+        <v>40909</v>
+      </c>
+      <c r="F651" t="n">
+        <v>100</v>
+      </c>
+      <c r="G651" t="n">
+        <v>100</v>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="K651" t="inlineStr"/>
+      <c r="M651" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C652" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>United Kingdom: Flood - 01/01/2012</t>
+        </is>
+      </c>
+      <c r="E652" s="1" t="n">
+        <v>40909</v>
+      </c>
+      <c r="F652" t="n">
+        <v>100</v>
+      </c>
+      <c r="G652" t="n">
+        <v>100</v>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="K652" t="inlineStr"/>
+      <c r="M652" t="inlineStr"/>
+    </row>
     <row r="2176">
       <c r="A2176" t="inlineStr">
         <is>
@@ -1878,6 +2246,59 @@
       </c>
       <c r="M5294" t="inlineStr"/>
     </row>
+    <row r="5355">
+      <c r="A5355" t="inlineStr">
+        <is>
+          <t>TUR</t>
+        </is>
+      </c>
+      <c r="B5355" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C5355" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D5355" t="inlineStr">
+        <is>
+          <t>Turkey: Landslide risk evacuations - Çaybaşı district (ORDU)  - 12/08/2018</t>
+        </is>
+      </c>
+      <c r="E5355" s="1" t="n">
+        <v>43324</v>
+      </c>
+      <c r="F5355" t="n">
+        <v>78</v>
+      </c>
+      <c r="G5355" t="n">
+        <v>78</v>
+      </c>
+      <c r="H5355" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I5355" t="inlineStr">
+        <is>
+          <t>Mass Movement</t>
+        </is>
+      </c>
+      <c r="J5355" t="inlineStr">
+        <is>
+          <t>Landslide/Wet mass movement</t>
+        </is>
+      </c>
+      <c r="K5355" t="inlineStr"/>
+      <c r="L5355" t="n">
+        <v>3517</v>
+      </c>
+      <c r="M5355" t="inlineStr">
+        <is>
+          <t>Displacement without preventive evacuations reported</t>
+        </is>
+      </c>
+    </row>
     <row r="5623">
       <c r="A5623" t="inlineStr">
         <is>
@@ -1984,6 +2405,112 @@
         </is>
       </c>
     </row>
+    <row r="6299">
+      <c r="A6299" t="inlineStr">
+        <is>
+          <t>MMR</t>
+        </is>
+      </c>
+      <c r="B6299" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="C6299" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D6299" t="inlineStr">
+        <is>
+          <t>Myanmar: Riverbank erosion - Maubin; Nyaungdon townships; Maubin district; Ayeyarwady Region - 01/01/2019</t>
+        </is>
+      </c>
+      <c r="E6299" s="1" t="n">
+        <v>43475</v>
+      </c>
+      <c r="F6299" t="n">
+        <v>16</v>
+      </c>
+      <c r="G6299" t="n">
+        <v>16</v>
+      </c>
+      <c r="H6299" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I6299" t="inlineStr">
+        <is>
+          <t>Mass Movement</t>
+        </is>
+      </c>
+      <c r="J6299" t="inlineStr">
+        <is>
+          <t>Landslide/Wet mass movement</t>
+        </is>
+      </c>
+      <c r="K6299" t="inlineStr"/>
+      <c r="L6299" t="n">
+        <v>3819</v>
+      </c>
+      <c r="M6299" t="inlineStr">
+        <is>
+          <t>Displacement without preventive evacuations reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="6842">
+      <c r="A6842" t="inlineStr">
+        <is>
+          <t>NIC</t>
+        </is>
+      </c>
+      <c r="B6842" t="inlineStr">
+        <is>
+          <t>Nicaragua</t>
+        </is>
+      </c>
+      <c r="C6842" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D6842" t="inlineStr">
+        <is>
+          <t>Nicaragua: Evacuated - Carazo, Rivas, San Rafael del Sur and Boaco - 22/05/2019</t>
+        </is>
+      </c>
+      <c r="E6842" s="1" t="n">
+        <v>43607</v>
+      </c>
+      <c r="F6842" t="n">
+        <v>67</v>
+      </c>
+      <c r="G6842" t="n">
+        <v>67</v>
+      </c>
+      <c r="H6842" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I6842" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="J6842" t="inlineStr">
+        <is>
+          <t>Flood</t>
+        </is>
+      </c>
+      <c r="K6842" t="inlineStr"/>
+      <c r="L6842" t="n">
+        <v>5179</v>
+      </c>
+      <c r="M6842" t="inlineStr">
+        <is>
+          <t>Displacement without preventive evacuations reported</t>
+        </is>
+      </c>
+    </row>
     <row r="7431">
       <c r="A7431" t="inlineStr">
         <is>
@@ -2032,6 +2559,59 @@
         <v>6340</v>
       </c>
       <c r="M7431" t="inlineStr">
+        <is>
+          <t>Displacement reporting preventive evacuations</t>
+        </is>
+      </c>
+    </row>
+    <row r="8720">
+      <c r="A8720" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="B8720" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C8720" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D8720" t="inlineStr">
+        <is>
+          <t>Sri Lanka: Risk of Landslide - Central (Kandy/Ganga ihala korale) - 01/07/2020</t>
+        </is>
+      </c>
+      <c r="E8720" s="1" t="n">
+        <v>44013</v>
+      </c>
+      <c r="F8720" t="n">
+        <v>70</v>
+      </c>
+      <c r="G8720" t="n">
+        <v>70</v>
+      </c>
+      <c r="H8720" t="inlineStr">
+        <is>
+          <t>Weather related</t>
+        </is>
+      </c>
+      <c r="I8720" t="inlineStr">
+        <is>
+          <t>Mass Movement</t>
+        </is>
+      </c>
+      <c r="J8720" t="inlineStr">
+        <is>
+          <t>Landslide/Wet mass movement</t>
+        </is>
+      </c>
+      <c r="K8720" t="inlineStr"/>
+      <c r="L8720" t="n">
+        <v>7761</v>
+      </c>
+      <c r="M8720" t="inlineStr">
         <is>
           <t>Displacement reporting preventive evacuations</t>
         </is>

</xml_diff>